<commit_message>
feat(Imports): Achats: ajoute les nouveaux formats d'imports (#6841)
</commit_message>
<xml_diff>
--- a/api/tests/files/achats/purchases_good.xlsx
+++ b/api/tests/files/achats/purchases_good.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="purchases_good" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="purchases_good_xlsx_source" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t xml:space="preserve">siret</t>
   </si>
@@ -40,7 +40,16 @@
     <t xml:space="preserve">famille_produits</t>
   </si>
   <si>
-    <t xml:space="preserve">caracteristiques</t>
+    <t xml:space="preserve">categories_egalim</t>
+  </si>
+  <si>
+    <t xml:space="preserve">origine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">est_circuit_court</t>
+  </si>
+  <si>
+    <t xml:space="preserve">est_local</t>
   </si>
   <si>
     <t xml:space="preserve">definition_local</t>
@@ -49,22 +58,22 @@
     <t xml:space="preserve">Pommes, rouges, local</t>
   </si>
   <si>
-    <t xml:space="preserve">Le bon traiteur </t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025-01-02</t>
+    <t xml:space="preserve">Le bon traiteur</t>
   </si>
   <si>
     <t xml:space="preserve">90.11</t>
   </si>
   <si>
-    <t xml:space="preserve"> PRODUITS_LAITIERS </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BIO, LOCAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> DEPARTEMENT</t>
+    <t xml:space="preserve">PRODUITS_LAITIERS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BIO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DEPARTEMENT</t>
   </si>
 </sst>
 </file>
@@ -73,14 +82,13 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="@"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
   <fonts count="4">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -145,7 +153,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -272,67 +280,84 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="13.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="6.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="1" width="20.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="6.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="19.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="6.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="8.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="13.34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="0" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="0" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="0" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="0" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="0" t="s">
         <v>7</v>
+      </c>
+      <c r="I1" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="0" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="0" t="n">
         <v>21010034300016</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="1" t="s">
+      <c r="B2" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="C2" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="D2" s="1" t="n">
+        <v>44683</v>
+      </c>
+      <c r="E2" s="0" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="F2" s="0" t="s">
         <v>14</v>
+      </c>
+      <c r="G2" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="J2" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="K2" s="0" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ajout de definition_local_km aux nouveaux imports
</commit_message>
<xml_diff>
--- a/api/tests/files/achats/purchases_good.xlsx
+++ b/api/tests/files/achats/purchases_good.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t xml:space="preserve">siret</t>
   </si>
@@ -53,6 +53,9 @@
   </si>
   <si>
     <t xml:space="preserve">definition_local</t>
+  </si>
+  <si>
+    <t xml:space="preserve">definition_local_km</t>
   </si>
   <si>
     <t xml:space="preserve">Pommes, rouges, local</t>
@@ -89,6 +92,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -148,12 +152,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -177,37 +185,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -280,84 +288,87 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:L2"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="6.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="19.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="6.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="8.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="13.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="13.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="6.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="19.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="16.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="6.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="8.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="13.34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="0" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="0" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
+      </c>
+      <c r="L1" s="0" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>21010034300016</v>
       </c>
-      <c r="B2" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="1" t="n">
+      <c r="C2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="2" t="n">
         <v>44683</v>
       </c>
-      <c r="E2" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" s="0" t="s">
+      <c r="E2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="F2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J2" s="0" t="s">
+      <c r="G2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="K2" s="0" t="s">
+      <c r="J2" s="1" t="s">
         <v>17</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor(Imports): Achats: màj suite à la modification des valeurs dans definition_local & l'ajout de definition_local_km (#6849)
</commit_message>
<xml_diff>
--- a/api/tests/files/achats/purchases_good.xlsx
+++ b/api/tests/files/achats/purchases_good.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t xml:space="preserve">siret</t>
   </si>
@@ -53,6 +53,9 @@
   </si>
   <si>
     <t xml:space="preserve">definition_local</t>
+  </si>
+  <si>
+    <t xml:space="preserve">definition_local_km</t>
   </si>
   <si>
     <t xml:space="preserve">Pommes, rouges, local</t>
@@ -89,6 +92,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -148,12 +152,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -177,37 +185,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -280,84 +288,87 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:L2"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="6.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="19.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="6.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="8.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="13.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="13.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="6.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="19.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="16.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="6.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="8.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="13.34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="0" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="0" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
+      </c>
+      <c r="L1" s="0" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>21010034300016</v>
       </c>
-      <c r="B2" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="1" t="n">
+      <c r="C2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="2" t="n">
         <v>44683</v>
       </c>
-      <c r="E2" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" s="0" t="s">
+      <c r="E2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="F2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J2" s="0" t="s">
+      <c r="G2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="K2" s="0" t="s">
+      <c r="J2" s="1" t="s">
         <v>17</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>